<commit_message>
feat(F-NAR-016): TREE-DIF-009 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-009.xlsx
+++ b/stories/arbres/TREE-DIF-009.xlsx
@@ -1197,12 +1197,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sous le plancher, les joints font tic, puis tac. Le wagon sent l'orange, encore un peu. Un ticket dépasse de la poche de papa. Dehors, un champ passe, tout vert. Le filet à bagages tremble, tout bas. Tu entends les rails, Amir ? Ils chantent. Le grand train va loin, ce matin. Nina pose un sac de toile, près des genoux. Dedans, des rails de bois s'entrechoquent. Je veux un petit train, comme le grand. Tu le poses où, alors ? Près des rails, avec Nina. Les pièces sont dans le sac. En ce moment, Amir sort une locomotive en bois. Elle est petite, toute lisse. J'ai les rails. On fait une longue voie. Jaune, bleu, ou rouge ?</t>
+          <t>Sous le plancher, les joints font tic, puis tac. Tu entends les rails, Amir ? Ils chantent. Le wagon sent l'orange, encore un peu. Un ticket dépasse de la poche de papa, sous le filet. Le grand train va loin, ce matin. Dehors, un champ passe, tout vert, derrière la vitre. Nina pose un sac de toile, près des genoux. Dedans, des rails de bois s'entrechoquent. Je veux un petit train, comme le grand. Tu le poses où, alors ? Près des rails, avec Nina. Les pièces sont dans le sac. En ce moment, Amir sort une locomotive en bois. Elle est petite, toute lisse. J'ai les rails. On fait une longue voie. Jaune, bleu, ou rouge ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sous le plancher, les joints font tic, puis tac. Le wagon sent l'orange, encore un peu. Un ticket dépasse de la poche de papa. Dehors, un champ passe, tout vert. Le filet à bagages tremble, tout bas. Tu entends les rails, Amir ? Ils chantent. Le grand train va loin, ce matin. Nina pose un sac de toile, près des genoux. Dedans, des rails de bois s'entrechoquent. Je veux un petit train, comme le grand. Tu le poses où, alors ? Près des rails, avec Nina. Les pièces sont dans le sac. En ce moment, Amir sort une locomotive en bois. Elle est petite, toute lisse. J'ai les rails. On fait une longue voie. Jaune, bleu, ou rouge ?</t>
+          <t>Sous le plancher, les joints font tic, puis tac. Tu entends les rails, Amir ? Ils chantent. Le wagon sent l'orange, encore un peu. Un ticket dépasse de la poche de papa, sous le filet. Le grand train va loin, ce matin. Dehors, un champ passe, tout vert, derrière la vitre. Nina pose un sac de toile, près des genoux. Dedans, des rails de bois s'entrechoquent. Je veux un petit train, comme le grand. Tu le poses où, alors ? Près des rails, avec Nina. Les pièces sont dans le sac. En ce moment, Amir sort une locomotive en bois. Elle est petite, toute lisse. J'ai les rails. On fait une longue voie. Jaune, bleu, ou rouge ?</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1338,13 +1338,12 @@
       <c r="AW2" t="inlineStr">
         <is>
           <t>narrateur|Sous le plancher, les joints font tic, puis tac.
-narrateur|Le wagon sent l'orange, encore un peu.
-narrateur|Un ticket dépasse de la poche de papa.
-narrateur|Dehors, un champ passe, tout vert.
-narrateur|Le filet à bagages tremble, tout bas.
 papa|Tu entends les rails, Amir ?
 enfant-m|Ils chantent.
+narrateur|Le wagon sent l'orange, encore un peu.
+narrateur|Un ticket dépasse de la poche de papa, sous le filet.
 maman|Le grand train va loin, ce matin.
+narrateur|Dehors, un champ passe, tout vert, derrière la vitre.
 narrateur|Nina pose un sac de toile, près des genoux.
 narrateur|Dedans, des rails de bois s'entrechoquent.
 enfant-m|Je veux un petit train, comme le grand.
@@ -2307,12 +2306,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Amir pose un pont de bois au-dessus de l'ombre. Les pieds du pont touchent le plancher jaune. Le haut est trop loin. Tes bras sont plus courts, c'est tout. Nina tend les siens, jusqu'à la planche. Je tiens le milieu, moi. Moi, les pieds. Vous le tenez, chacun un bout. Le pont tremble un peu, puis tient.</t>
+          <t>Amir pose un pont de bois au-dessus de l'ombre. Les pieds du pont touchent le plancher jaune. Le haut est trop loin. La planche est un peu haute. Nina tend les siens, jusqu'à la planche. Je tiens le milieu, moi. Moi, les pieds. Vous le tenez, chacun un bout. Le pont tremble un peu, puis tient.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Amir pose un pont de bois au-dessus de l'ombre. Les pieds du pont touchent le plancher jaune. Le haut est trop loin. Tes bras sont plus courts, c'est tout. Nina tend les siens, jusqu'à la planche. Je tiens le milieu, moi. Moi, les pieds. Vous le tenez, chacun un bout. Le pont tremble un peu, puis tient.</t>
+          <t>Amir pose un pont de bois au-dessus de l'ombre. Les pieds du pont touchent le plancher jaune. Le haut est trop loin. La planche est un peu haute. Nina tend les siens, jusqu'à la planche. Je tiens le milieu, moi. Moi, les pieds. Vous le tenez, chacun un bout. Le pont tremble un peu, puis tient.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2450,7 +2449,7 @@
           <t>narrateur|Amir pose un pont de bois au-dessus de l'ombre.
 narrateur|Les pieds du pont touchent le plancher jaune.
 enfant-m|Le haut est trop loin.
-papa|Tes bras sont plus courts, c'est tout.
+papa|La planche est un peu haute.
 narrateur|Nina tend les siens, jusqu'à la planche.
 enfant-f|Je tiens le milieu, moi.
 enfant-m|Moi, les pieds.
@@ -4791,12 +4790,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sous les sièges. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sous les sièges. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sous les sièges. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sous les sièges. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4936,7 +4935,7 @@
 enfant-f|Moi, je garde le toit.
 narrateur|La locomotive roule, puis touche la pierre.
 maman|Elle s'arrête sous les sièges.
-papa|Deux hauteurs, un seul train.
+papa|Le galet l'a retenue.
 enfant-m|Elle est à la gare.</t>
         </is>
       </c>
@@ -9766,12 +9765,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête le long de la vitre. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête le long de la vitre. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête le long de la vitre. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête le long de la vitre. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9911,7 +9910,7 @@
 enfant-f|Moi, je garde le toit.
 narrateur|La locomotive roule, puis touche la pierre.
 maman|Elle s'arrête le long de la vitre.
-papa|Deux hauteurs, un seul train.
+papa|Le galet l'a retenue.
 enfant-m|Elle est à la gare.</t>
         </is>
       </c>
@@ -14737,12 +14736,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sur la valise. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sur la valise. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sur la valise. Deux hauteurs, un seul train. Elle est à la gare.</t>
+          <t>Le galet, pour arrêter. Amir le pose au quai, tout près du sol. Moi, je garde le toit. La locomotive roule, puis touche la pierre. Elle s'arrête sur la valise. Le galet l'a retenue. Elle est à la gare.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14882,7 +14881,7 @@
 enfant-f|Moi, je garde le toit.
 narrateur|La locomotive roule, puis touche la pierre.
 maman|Elle s'arrête sur la valise.
-papa|Deux hauteurs, un seul train.
+papa|Le galet l'a retenue.
 enfant-m|Elle est à la gare.</t>
         </is>
       </c>
@@ -16487,7 +16486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16593,6 +16592,13 @@
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish TREE-DIF-009 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-009.xlsx
+++ b/stories/arbres/TREE-DIF-009.xlsx
@@ -4631,17 +4631,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>La plume, sur le toit. Nina glisse la plume au faîte, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près.</t>
+          <t>La plume, sur le toit. Nina glisse la plume au toit, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, sur le toit. Nina glisse la plume au faîte, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, sur le toit. Nina glisse la plume au toit, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, sur le toit. Nina glisse la plume au faîte, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près. [pause]</t>
+          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, sur le toit. Nina glisse la plume au toit, haute. Amir pousse depuis le plancher, lent. Je la vois. La plume tremble, puis s'arrête. Le train s'aligne sous le blanc. Deux hauteurs tiennent la gare. Vous l'avez posé, chacun son bout. L'éclat de ticket se loge sous la plume. Le pied de la chaise est tout près. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4776,7 +4776,7 @@
       <c r="AW20" t="inlineStr">
         <is>
           <t>enfant-m|La plume, sur le toit.
-narrateur|Nina glisse la plume au faîte, haute.
+narrateur|Nina glisse la plume au toit, haute.
 narrateur|Amir pousse depuis le plancher, lent.
 enfant-f|Je la vois.
 narrateur|La plume tremble, puis s'arrête.
@@ -4816,17 +4816,17 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'éclat de ticket se loge sous la plume du faîte.</t>
+          <t>Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'éclat de ticket se loge sous la plume du toit.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du faîte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du toit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du faîte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le toit a failli rester trop haut. Le petit train s'aligne sous la chaise, sous la plume. Je l'ai posée. Moi, j'ai poussé. Chacun son bout, chacun sa hauteur. Le quai jaune touche presque le pied. Les grands rails chantent, tout bas. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du toit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr"/>
@@ -4971,7 +4971,7 @@
 papa|Chacun son bout, chacun sa hauteur.
 maman|Le quai jaune touche presque le pied.
 narrateur|Les grands rails chantent, tout bas.
-narrateur|L'éclat de ticket se loge sous la plume du faîte.</t>
+narrateur|L'éclat de ticket se loge sous la plume du toit.</t>
         </is>
       </c>
       <c r="AX21" t="inlineStr">
@@ -9541,17 +9541,17 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Le grelot, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez hissé, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette.</t>
+          <t>Le grelot, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez monté, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt;, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez hissé, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;grelot&lt;/emphasis&gt;, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez monté, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;grelot&lt;/emphasis&gt;, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez hissé, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette. [pause]</t>
+          <t>Le &lt;emphasis&gt;grelot&lt;/emphasis&gt;, en haut. Nina pose le grelot sur le toit de gare. Amir pousse depuis le plancher, lent. Quand ça tinte, tu es prête. Le grelot tinte, trop haut pour lui. Nina reçoit le train, à sa hauteur. La gare des nuages n'est plus trop haute. Vous l'avez monté, chacun son étage. L'éclat de ticket tinte avec le grelot. La chaise est juste sous la tablette. [pause]</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -9692,7 +9692,7 @@
 narrateur|Le grelot tinte, trop haut pour lui.
 narrateur|Nina reçoit le train, à sa hauteur.
 narrateur|La gare des nuages n'est plus trop haute.
-maman|Vous l'avez hissé, chacun son étage.
+maman|Vous l'avez monté, chacun son étage.
 narrateur|L'éclat de ticket tinte avec le grelot.
 papa|La chaise est juste sous la tablette.</t>
         </is>
@@ -9726,17 +9726,17 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>La gare a failli rester trop haute. Le petit train est sous la chaise, hissé au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'éclat de ticket tinte, caché sous le grelot du toit.</t>
+          <t>La gare a failli rester trop haute. Le petit train est sous la chaise, monté au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'éclat de ticket tinte, caché sous le grelot du toit.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La gare a failli rester trop haute. Le petit train est sous la chaise, hissé au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; tinte, caché sous le grelot du toit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La gare a failli rester trop haute. Le petit train est sous la chaise, monté au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; tinte, caché sous le grelot du toit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La gare a failli rester trop haute. Le petit train est sous la chaise, hissé au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; tinte, caché sous le grelot du toit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La gare a failli rester trop haute. Le petit train est sous la chaise, monté au tintement. Tu étais en haut. J'ai entendu. Le grelot a parlé d'un étage à l'autre. La tablette froide est devenue un quai. Les grands rails chantent, sous les nuages. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; tinte, caché sous le grelot du toit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
@@ -9875,7 +9875,7 @@
       <c r="AW47" t="inlineStr">
         <is>
           <t>narrateur|La gare a failli rester trop haute.
-narrateur|Le petit train est sous la chaise, hissé au tintement.
+narrateur|Le petit train est sous la chaise, monté au tintement.
 enfant-m|Tu étais en haut.
 enfant-f|J'ai entendu.
 papa|Le grelot a parlé d'un étage à l'autre.
@@ -9913,17 +9913,17 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>La plume, pour le ciel. Nina plante la plume au faîte, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette.</t>
+          <t>La plume, pour le ciel. Nina plante la plume au toit, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, pour le ciel. Nina plante la plume au faîte, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, pour le ciel. Nina plante la plume au toit, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, pour le ciel. Nina plante la plume au faîte, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette. [pause]</t>
+          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, pour le ciel. Nina plante la plume au toit, contre le verre. Amir vise le blanc, d'en bas. C'est ici. Le train grimpe, lent, vers la plume. Deux hauteurs se rejoignent au quai. Le ciel pâle reste collé au toit. Vous l'avez visé, de loin. L'éclat de ticket se loge sous la plume. Le pied de la chaise touche la tablette. [pause]</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
@@ -10058,7 +10058,7 @@
       <c r="AW48" t="inlineStr">
         <is>
           <t>enfant-m|La plume, pour le ciel.
-narrateur|Nina plante la plume au faîte, contre le verre.
+narrateur|Nina plante la plume au toit, contre le verre.
 narrateur|Amir vise le blanc, d'en bas.
 enfant-f|C'est ici.
 narrateur|Le train grimpe, lent, vers la plume.
@@ -10098,17 +10098,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'éclat de ticket se loge sous la plume du faîte bleu.</t>
+          <t>Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'éclat de ticket se loge sous la plume du toit bleu.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du faîte bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du toit bleu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du faîte bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le ciel a failli cacher le quai. Le petit train s'aligne sous la chaise, sous la plume. C'était ici. Je visais le blanc. Deux hauteurs ont visé le même toit. Le verre garde un fil de plume. Les grands rails chantent, contre le ciel. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; se loge sous la plume du toit bleu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10253,7 +10253,7 @@
 papa|Deux hauteurs ont visé le même toit.
 maman|Le verre garde un fil de plume.
 narrateur|Les grands rails chantent, contre le ciel.
-narrateur|L'éclat de ticket se loge sous la plume du faîte bleu.</t>
+narrateur|L'éclat de ticket se loge sous la plume du toit bleu.</t>
         </is>
       </c>
       <c r="AX49" t="inlineStr">
@@ -10285,17 +10285,17 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Le galet, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez hissé, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains.</t>
+          <t>Le galet, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez monté, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;galet&lt;/emphasis&gt;, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez hissé, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;galet&lt;/emphasis&gt;, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez monté, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;galet&lt;/emphasis&gt;, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez hissé, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains. [pause]</t>
+          <t>Le &lt;emphasis&gt;galet&lt;/emphasis&gt;, pour pas reculer. Amir cale le galet derrière les roues. Nina tire le train, d'en haut, douce. Je pousse, toi tu tires. Le galet empêche de redescendre. Le train gagne le quai, lent. La tablette froide devient une gare. Vous l'avez monté, sans le lâcher. L'éclat de ticket reste derrière le galet. La chaise est là, sous vos mains. [pause]</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
@@ -10436,7 +10436,7 @@
 narrateur|Le galet empêche de redescendre.
 narrateur|Le train gagne le quai, lent.
 narrateur|La tablette froide devient une gare.
-maman|Vous l'avez hissé, sans le lâcher.
+maman|Vous l'avez monté, sans le lâcher.
 narrateur|L'éclat de ticket reste derrière le galet.
 papa|La chaise est là, sous vos mains.</t>
         </is>
@@ -13687,17 +13687,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>La plume, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train gravit la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente.</t>
+          <t>La plume, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train monte la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train gravit la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La &lt;emphasis level="moderate"&gt;plume&lt;/emphasis&gt;, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train monte la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train gravit la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente. [pause]</t>
+          <t>La &lt;emphasis&gt;plume&lt;/emphasis&gt;, sur la poignée. Nina plante la plume, tout en haut. Amir vise le blanc, depuis le tapis. Monte. Le train monte la pente, sous la plume. La fermeture reste close, sans danser. Deux hauteurs tiennent le pont de tissu. Vous l'avez visé, de la poignée au tapis. L'éclat de ticket se colle à la plume. La chaise attend, après la descente. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13835,7 +13835,7 @@
 narrateur|Nina plante la plume, tout en haut.
 narrateur|Amir vise le blanc, depuis le tapis.
 enfant-f|Monte.
-narrateur|Le train gravit la pente, sous la plume.
+narrateur|Le train monte la pente, sous la plume.
 narrateur|La fermeture reste close, sans danser.
 narrateur|Deux hauteurs tiennent le pont de tissu.
 maman|Vous l'avez visé, de la poignée au tapis.
@@ -13872,17 +13872,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au faîte. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'éclat de ticket voyage, collé à la plume de poignée.</t>
+          <t>La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au toit. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'éclat de ticket voyage, collé à la plume de poignée.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au faîte. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; voyage, collé à la plume de poignée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au toit. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'&lt;emphasis level="moderate"&gt;éclat de ticket&lt;/emphasis&gt; voyage, collé à la plume de poignée.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au faîte. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; voyage, collé à la plume de poignée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La poignée a failli rester trop loin. Le petit train arrive sous la chaise, plume au toit. Monte, j'ai dit. J'ai visé. Le blanc a relié le tapis à la poignée. Le tissu rêche garde un fil de plume. Les grands rails chantent, sous la valise. L'&lt;emphasis&gt;éclat de ticket&lt;/emphasis&gt; voyage, collé à la plume de poignée.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -14021,7 +14021,7 @@
       <c r="AW69" t="inlineStr">
         <is>
           <t>narrateur|La poignée a failli rester trop loin.
-narrateur|Le petit train arrive sous la chaise, plume au faîte.
+narrateur|Le petit train arrive sous la chaise, plume au toit.
 enfant-f|Monte, j'ai dit.
 enfant-m|J'ai visé.
 papa|Le blanc a relié le tapis à la poignée.
@@ -17439,7 +17439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17559,6 +17559,13 @@
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>